<commit_message>
Move images to figures
</commit_message>
<xml_diff>
--- a/gantt/Gantt Chart.xlsx
+++ b/gantt/Gantt Chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr saveExternalLinkValues="0" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferry\Desktop\UPC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ferry\Projects\ALS1\gantt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB17D755-AF9A-4787-BD33-656DC3976464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAAEE09D-BF98-4B08-BE34-DDB45127A726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{810C8B86-46A3-44F4-9DF3-DC25E25C8DFC}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <r>
       <rPr>
@@ -83,12 +83,27 @@
       <t xml:space="preserve"> </t>
     </r>
   </si>
+  <si>
+    <t>TASK TITLE</t>
+  </si>
+  <si>
+    <t>Project Management &amp; Setup</t>
+  </si>
+  <si>
+    <t>Repository creation and structure</t>
+  </si>
+  <si>
+    <t>TASK OWNER</t>
+  </si>
+  <si>
+    <t>Ferran and Noa</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -124,18 +139,124 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="8">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="double">
+        <color theme="2" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color theme="2" tint="-0.499984740745262"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -147,7 +268,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -157,6 +278,49 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -474,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9811F35A-BD43-4094-ACEF-D2015FF5FE77}">
-  <dimension ref="B3:J4"/>
+  <dimension ref="B3:J9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
@@ -503,10 +667,55 @@
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
     </row>
+    <row r="6" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="11"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="17" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="7">
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B6:D7"/>
+    <mergeCell ref="E6:G7"/>
+    <mergeCell ref="E8:G8"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="B4:J4"/>
+    <mergeCell ref="B8:D8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -514,15 +723,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010045689DC494B23342B7923C92B2C5978C" ma:contentTypeVersion="0" ma:contentTypeDescription="Crea un document nou" ma:contentTypeScope="" ma:versionID="fd111a9c02607776e4be7964bd45a281">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4086592f9e68471b8ffacb66d88183bc">
     <xsd:element name="properties">
@@ -636,6 +836,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -643,14 +852,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFACF0AE-1A74-4646-9DBB-C0D55DD8BB2C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45720B53-44F7-44AB-9F56-E2F827957C3C}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -662,6 +863,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FFACF0AE-1A74-4646-9DBB-C0D55DD8BB2C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>